<commit_message>
Daily pricing refresh 2026-06-16
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.86/GPU/hr (₹81) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-17
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-19
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15225,10 +15225,10 @@
         </is>
       </c>
       <c r="U199" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V199" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W199" s="9" t="n"/>
       <c r="X199" s="8" t="n"/>
@@ -15238,7 +15238,7 @@
         </is>
       </c>
       <c r="Z199" s="14" t="n">
-        <v>1.151</v>
+        <v>0.868</v>
       </c>
       <c r="AA199" s="10" t="inlineStr">
         <is>
@@ -16377,16 +16377,16 @@
         </is>
       </c>
       <c r="U215" s="11" t="n">
-        <v>0.731</v>
+        <v>0.84</v>
       </c>
       <c r="V215" s="12" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="W215" s="6" t="n">
-        <v>3202</v>
+        <v>3679</v>
       </c>
       <c r="X215" s="12" t="n">
-        <v>302920</v>
+        <v>348089</v>
       </c>
       <c r="Y215" s="3" t="inlineStr">
         <is>
@@ -16394,7 +16394,7 @@
         </is>
       </c>
       <c r="Z215" s="14" t="n">
-        <v>0.556</v>
+        <v>0.354</v>
       </c>
       <c r="AA215" s="10" t="inlineStr">
         <is>
@@ -18129,16 +18129,16 @@
         </is>
       </c>
       <c r="U239" s="11" t="n">
-        <v>0.748</v>
+        <v>0.86</v>
       </c>
       <c r="V239" s="12" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="W239" s="6" t="n">
-        <v>19657</v>
+        <v>22601</v>
       </c>
       <c r="X239" s="12" t="n">
-        <v>1859790</v>
+        <v>2138262</v>
       </c>
       <c r="Y239" s="3" t="inlineStr">
         <is>
@@ -18146,7 +18146,7 @@
         </is>
       </c>
       <c r="Z239" s="14" t="n">
-        <v>0.243</v>
+        <v>0.081</v>
       </c>
       <c r="AA239" s="10" t="inlineStr">
         <is>
@@ -32809,10 +32809,10 @@
         </is>
       </c>
       <c r="U439" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V439" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W439" s="9" t="n"/>
       <c r="X439" s="8" t="n"/>
@@ -32822,7 +32822,7 @@
         </is>
       </c>
       <c r="Z439" s="14" t="n">
-        <v>1.151</v>
+        <v>0.868</v>
       </c>
       <c r="AA439" s="10" t="inlineStr">
         <is>
@@ -33961,16 +33961,16 @@
         </is>
       </c>
       <c r="U455" s="11" t="n">
-        <v>0.731</v>
+        <v>0.84</v>
       </c>
       <c r="V455" s="12" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="W455" s="6" t="n">
-        <v>3202</v>
+        <v>3679</v>
       </c>
       <c r="X455" s="12" t="n">
-        <v>302920</v>
+        <v>348089</v>
       </c>
       <c r="Y455" s="3" t="inlineStr">
         <is>
@@ -33978,7 +33978,7 @@
         </is>
       </c>
       <c r="Z455" s="14" t="n">
-        <v>0.556</v>
+        <v>0.354</v>
       </c>
       <c r="AA455" s="10" t="inlineStr">
         <is>
@@ -35713,16 +35713,16 @@
         </is>
       </c>
       <c r="U479" s="11" t="n">
-        <v>0.748</v>
+        <v>0.86</v>
       </c>
       <c r="V479" s="12" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="W479" s="6" t="n">
-        <v>19657</v>
+        <v>22601</v>
       </c>
       <c r="X479" s="12" t="n">
-        <v>1859790</v>
+        <v>2138262</v>
       </c>
       <c r="Y479" s="3" t="inlineStr">
         <is>
@@ -35730,7 +35730,7 @@
         </is>
       </c>
       <c r="Z479" s="14" t="n">
-        <v>0.243</v>
+        <v>0.081</v>
       </c>
       <c r="AA479" s="10" t="inlineStr">
         <is>
@@ -50393,10 +50393,10 @@
         </is>
       </c>
       <c r="U679" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V679" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W679" s="9" t="n"/>
       <c r="X679" s="8" t="n"/>
@@ -50406,7 +50406,7 @@
         </is>
       </c>
       <c r="Z679" s="14" t="n">
-        <v>1.151</v>
+        <v>0.868</v>
       </c>
       <c r="AA679" s="10" t="inlineStr">
         <is>
@@ -51541,16 +51541,16 @@
         </is>
       </c>
       <c r="U695" s="11" t="n">
-        <v>0.731</v>
+        <v>0.84</v>
       </c>
       <c r="V695" s="12" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="W695" s="6" t="n">
-        <v>3202</v>
+        <v>3679</v>
       </c>
       <c r="X695" s="12" t="n">
-        <v>302920</v>
+        <v>348089</v>
       </c>
       <c r="Y695" s="3" t="inlineStr">
         <is>
@@ -51558,7 +51558,7 @@
         </is>
       </c>
       <c r="Z695" s="14" t="n">
-        <v>0.556</v>
+        <v>0.354</v>
       </c>
       <c r="AA695" s="10" t="inlineStr">
         <is>
@@ -53293,16 +53293,16 @@
         </is>
       </c>
       <c r="U719" s="11" t="n">
-        <v>0.748</v>
+        <v>0.86</v>
       </c>
       <c r="V719" s="12" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="W719" s="6" t="n">
-        <v>19657</v>
+        <v>22601</v>
       </c>
       <c r="X719" s="12" t="n">
-        <v>1859790</v>
+        <v>2138262</v>
       </c>
       <c r="Y719" s="3" t="inlineStr">
         <is>
@@ -53310,7 +53310,7 @@
         </is>
       </c>
       <c r="Z719" s="14" t="n">
-        <v>0.243</v>
+        <v>0.081</v>
       </c>
       <c r="AA719" s="10" t="inlineStr">
         <is>
@@ -61011,10 +61011,10 @@
         </is>
       </c>
       <c r="U823" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V823" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W823" s="9" t="n"/>
       <c r="X823" s="8" t="n"/>
@@ -62147,16 +62147,16 @@
         </is>
       </c>
       <c r="U839" s="11" t="n">
-        <v>0.731</v>
+        <v>0.84</v>
       </c>
       <c r="V839" s="12" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="W839" s="6" t="n">
-        <v>3202</v>
+        <v>3679</v>
       </c>
       <c r="X839" s="12" t="n">
-        <v>302920</v>
+        <v>348089</v>
       </c>
       <c r="Y839" s="3" t="inlineStr">
         <is>
@@ -62164,7 +62164,7 @@
         </is>
       </c>
       <c r="Z839" s="14" t="n">
-        <v>0.154</v>
+        <v>0.005</v>
       </c>
       <c r="AA839" s="10" t="inlineStr">
         <is>
@@ -63899,16 +63899,16 @@
         </is>
       </c>
       <c r="U863" s="11" t="n">
-        <v>0.748</v>
+        <v>0.86</v>
       </c>
       <c r="V863" s="12" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="W863" s="6" t="n">
-        <v>19657</v>
+        <v>22601</v>
       </c>
       <c r="X863" s="12" t="n">
-        <v>1859790</v>
+        <v>2138262</v>
       </c>
       <c r="Y863" s="3" t="inlineStr">
         <is>
@@ -63916,7 +63916,7 @@
         </is>
       </c>
       <c r="Z863" s="13" t="n">
-        <v>-0.063</v>
+        <v>-0.185</v>
       </c>
       <c r="AA863" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-20
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-21
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-23
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-24
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-25
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-26
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-27
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-29
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-06-30
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-02
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-03
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-04
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-05
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-06
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-07
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-08
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -7789,10 +7789,10 @@
         </is>
       </c>
       <c r="U99" s="11" t="n">
-        <v>5.7211</v>
+        <v>6.8655</v>
       </c>
       <c r="V99" s="12" t="n">
-        <v>541</v>
+        <v>650</v>
       </c>
       <c r="W99" s="9" t="n"/>
       <c r="X99" s="8" t="n"/>
@@ -7802,7 +7802,7 @@
         </is>
       </c>
       <c r="Z99" s="13" t="n">
-        <v>-0.215</v>
+        <v>-0.346</v>
       </c>
       <c r="AA99" s="10" t="inlineStr"/>
     </row>
@@ -25369,10 +25369,10 @@
         </is>
       </c>
       <c r="U339" s="11" t="n">
-        <v>5.7211</v>
+        <v>6.8655</v>
       </c>
       <c r="V339" s="12" t="n">
-        <v>541</v>
+        <v>650</v>
       </c>
       <c r="W339" s="9" t="n"/>
       <c r="X339" s="8" t="n"/>
@@ -25382,7 +25382,7 @@
         </is>
       </c>
       <c r="Z339" s="13" t="n">
-        <v>-0.215</v>
+        <v>-0.346</v>
       </c>
       <c r="AA339" s="10" t="inlineStr"/>
     </row>
@@ -42949,10 +42949,10 @@
         </is>
       </c>
       <c r="U579" s="11" t="n">
-        <v>5.7211</v>
+        <v>6.8655</v>
       </c>
       <c r="V579" s="12" t="n">
-        <v>541</v>
+        <v>650</v>
       </c>
       <c r="W579" s="9" t="n"/>
       <c r="X579" s="8" t="n"/>
@@ -42962,7 +42962,7 @@
         </is>
       </c>
       <c r="Z579" s="13" t="n">
-        <v>-0.215</v>
+        <v>-0.346</v>
       </c>
       <c r="AA579" s="10" t="inlineStr"/>
     </row>
@@ -57175,10 +57175,10 @@
         </is>
       </c>
       <c r="U771" s="11" t="n">
-        <v>5.7211</v>
+        <v>6.8655</v>
       </c>
       <c r="V771" s="12" t="n">
-        <v>541</v>
+        <v>650</v>
       </c>
       <c r="W771" s="9" t="n"/>
       <c r="X771" s="8" t="n"/>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-10
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-12
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-13
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-14
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -54076,7 +54076,7 @@
       <c r="Z729" s="3" t="n"/>
       <c r="AA729" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -54636,7 +54636,7 @@
       <c r="Z737" s="3" t="n"/>
       <c r="AA737" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -55224,7 +55224,7 @@
       <c r="Z745" s="3" t="n"/>
       <c r="AA745" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -55812,7 +55812,7 @@
       <c r="Z753" s="3" t="n"/>
       <c r="AA753" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -56372,7 +56372,7 @@
       <c r="Z761" s="3" t="n"/>
       <c r="AA761" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -57016,7 +57016,7 @@
       <c r="Z769" s="3" t="n"/>
       <c r="AA769" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H100 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -57648,7 +57648,7 @@
       <c r="Z777" s="3" t="n"/>
       <c r="AA777" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -58208,7 +58208,7 @@
       <c r="Z785" s="3" t="n"/>
       <c r="AA785" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -58796,7 +58796,7 @@
       <c r="Z793" s="3" t="n"/>
       <c r="AA793" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -59384,7 +59384,7 @@
       <c r="Z801" s="3" t="n"/>
       <c r="AA801" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -59944,7 +59944,7 @@
       <c r="Z809" s="3" t="n"/>
       <c r="AA809" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -60560,7 +60560,7 @@
       <c r="Z817" s="3" t="n"/>
       <c r="AA817" s="10" t="inlineStr">
         <is>
-          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 128 vCPU, 1500GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
+          <t>Vultr does not offer H200 SXM. Nearest: L40S (L40S, 64 vCPU, 750GB RAM) at $1.56/GPU/hr (₹148) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -61123,13 +61123,13 @@
         </is>
       </c>
       <c r="O825" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P825" s="3" t="n">
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="Q825" s="3" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="R825" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-15
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-16
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="S52" s="3" t="inlineStr">
         <is>
-          <t>eastus</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T52" s="3" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="AA52" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -5673,24 +5673,24 @@
         </is>
       </c>
       <c r="U71" s="11" t="n">
-        <v>2.51</v>
+        <v>2.89</v>
       </c>
       <c r="V71" s="12" t="n">
-        <v>237</v>
+        <v>273</v>
       </c>
       <c r="W71" s="6" t="n">
-        <v>10994</v>
+        <v>12658</v>
       </c>
       <c r="X71" s="12" t="n">
-        <v>1040123</v>
+        <v>1197592</v>
       </c>
       <c r="Y71" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z71" s="14" t="n">
-        <v>0.112</v>
+      <c r="Z71" s="13" t="n">
+        <v>-0.035</v>
       </c>
       <c r="AA71" s="10" t="inlineStr">
         <is>
@@ -7465,16 +7465,16 @@
         </is>
       </c>
       <c r="U95" s="11" t="n">
-        <v>2.72</v>
+        <v>2.89</v>
       </c>
       <c r="V95" s="12" t="n">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="W95" s="6" t="n">
-        <v>71482</v>
+        <v>75949</v>
       </c>
       <c r="X95" s="12" t="n">
-        <v>6762874</v>
+        <v>7185554</v>
       </c>
       <c r="Y95" s="3" t="inlineStr">
         <is>
@@ -7482,7 +7482,7 @@
         </is>
       </c>
       <c r="Z95" s="13" t="n">
-        <v>-0.148</v>
+        <v>-0.198</v>
       </c>
       <c r="AA95" s="10" t="inlineStr">
         <is>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="S100" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>westus2</t>
         </is>
       </c>
       <c r="T100" s="3" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="AA100" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (westus2).</t>
         </is>
       </c>
     </row>
@@ -9289,16 +9289,16 @@
         </is>
       </c>
       <c r="U119" s="11" t="n">
-        <v>3.3</v>
+        <v>3.79</v>
       </c>
       <c r="V119" s="12" t="n">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="W119" s="6" t="n">
-        <v>14454</v>
+        <v>16600</v>
       </c>
       <c r="X119" s="12" t="n">
-        <v>1367493</v>
+        <v>1570545</v>
       </c>
       <c r="Y119" s="3" t="inlineStr">
         <is>
@@ -9306,7 +9306,7 @@
         </is>
       </c>
       <c r="Z119" s="13" t="n">
-        <v>-0.113</v>
+        <v>-0.228</v>
       </c>
       <c r="AA119" s="10" t="inlineStr">
         <is>
@@ -11053,16 +11053,16 @@
         </is>
       </c>
       <c r="U143" s="11" t="n">
-        <v>3.56</v>
+        <v>3.79</v>
       </c>
       <c r="V143" s="12" t="n">
-        <v>337</v>
+        <v>359</v>
       </c>
       <c r="W143" s="6" t="n">
-        <v>93557</v>
+        <v>99601</v>
       </c>
       <c r="X143" s="12" t="n">
-        <v>8851409</v>
+        <v>9423270</v>
       </c>
       <c r="Y143" s="3" t="inlineStr">
         <is>
@@ -11070,7 +11070,7 @@
         </is>
       </c>
       <c r="Z143" s="13" t="n">
-        <v>-0.317</v>
+        <v>-0.359</v>
       </c>
       <c r="AA143" s="10" t="inlineStr">
         <is>
@@ -12801,16 +12801,16 @@
         </is>
       </c>
       <c r="U167" s="11" t="n">
-        <v>0.33</v>
+        <v>0.39</v>
       </c>
       <c r="V167" s="12" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="W167" s="6" t="n">
-        <v>1445</v>
+        <v>1708</v>
       </c>
       <c r="X167" s="12" t="n">
-        <v>136749</v>
+        <v>161613</v>
       </c>
       <c r="Y167" s="3" t="inlineStr">
         <is>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="Z167" s="14" t="n">
-        <v>1.068</v>
+        <v>0.75</v>
       </c>
       <c r="AA167" s="10" t="inlineStr">
         <is>
@@ -14597,16 +14597,16 @@
         </is>
       </c>
       <c r="U191" s="11" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="V191" s="12" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="W191" s="6" t="n">
-        <v>8935</v>
+        <v>10249</v>
       </c>
       <c r="X191" s="12" t="n">
-        <v>845359</v>
+        <v>969677</v>
       </c>
       <c r="Y191" s="3" t="inlineStr">
         <is>
@@ -14614,7 +14614,7 @@
         </is>
       </c>
       <c r="Z191" s="14" t="n">
-        <v>0.64</v>
+        <v>0.43</v>
       </c>
       <c r="AA191" s="10" t="inlineStr">
         <is>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -16377,16 +16373,16 @@
         </is>
       </c>
       <c r="U215" s="11" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="V215" s="12" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="W215" s="6" t="n">
-        <v>3679</v>
+        <v>4336</v>
       </c>
       <c r="X215" s="12" t="n">
-        <v>348089</v>
+        <v>410248</v>
       </c>
       <c r="Y215" s="3" t="inlineStr">
         <is>
@@ -16394,7 +16390,7 @@
         </is>
       </c>
       <c r="Z215" s="14" t="n">
-        <v>0.354</v>
+        <v>0.149</v>
       </c>
       <c r="AA215" s="10" t="inlineStr">
         <is>
@@ -18129,24 +18125,24 @@
         </is>
       </c>
       <c r="U239" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V239" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W239" s="6" t="n">
-        <v>22601</v>
+        <v>26017</v>
       </c>
       <c r="X239" s="12" t="n">
-        <v>2138262</v>
+        <v>2461487</v>
       </c>
       <c r="Y239" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z239" s="14" t="n">
-        <v>0.081</v>
+      <c r="Z239" s="13" t="n">
+        <v>-0.061</v>
       </c>
       <c r="AA239" s="10" t="inlineStr">
         <is>
@@ -18351,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21839,7 +21835,7 @@
       </c>
       <c r="S292" s="3" t="inlineStr">
         <is>
-          <t>eastus</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T292" s="3" t="inlineStr">
@@ -21865,7 +21861,7 @@
       </c>
       <c r="AA292" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -23257,24 +23253,24 @@
         </is>
       </c>
       <c r="U311" s="11" t="n">
-        <v>2.51</v>
+        <v>2.89</v>
       </c>
       <c r="V311" s="12" t="n">
-        <v>237</v>
+        <v>273</v>
       </c>
       <c r="W311" s="6" t="n">
-        <v>10994</v>
+        <v>12658</v>
       </c>
       <c r="X311" s="12" t="n">
-        <v>1040123</v>
+        <v>1197592</v>
       </c>
       <c r="Y311" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z311" s="14" t="n">
-        <v>0.112</v>
+      <c r="Z311" s="13" t="n">
+        <v>-0.035</v>
       </c>
       <c r="AA311" s="10" t="inlineStr">
         <is>
@@ -25049,16 +25045,16 @@
         </is>
       </c>
       <c r="U335" s="11" t="n">
-        <v>2.72</v>
+        <v>2.89</v>
       </c>
       <c r="V335" s="12" t="n">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="W335" s="6" t="n">
-        <v>71482</v>
+        <v>75949</v>
       </c>
       <c r="X335" s="12" t="n">
-        <v>6762874</v>
+        <v>7185554</v>
       </c>
       <c r="Y335" s="3" t="inlineStr">
         <is>
@@ -25066,7 +25062,7 @@
         </is>
       </c>
       <c r="Z335" s="13" t="n">
-        <v>-0.148</v>
+        <v>-0.198</v>
       </c>
       <c r="AA335" s="10" t="inlineStr">
         <is>
@@ -25455,7 +25451,7 @@
       </c>
       <c r="S340" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>westus2</t>
         </is>
       </c>
       <c r="T340" s="3" t="inlineStr">
@@ -25481,7 +25477,7 @@
       </c>
       <c r="AA340" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (westus2).</t>
         </is>
       </c>
     </row>
@@ -26873,16 +26869,16 @@
         </is>
       </c>
       <c r="U359" s="11" t="n">
-        <v>3.3</v>
+        <v>3.79</v>
       </c>
       <c r="V359" s="12" t="n">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="W359" s="6" t="n">
-        <v>14454</v>
+        <v>16600</v>
       </c>
       <c r="X359" s="12" t="n">
-        <v>1367493</v>
+        <v>1570545</v>
       </c>
       <c r="Y359" s="3" t="inlineStr">
         <is>
@@ -26890,7 +26886,7 @@
         </is>
       </c>
       <c r="Z359" s="13" t="n">
-        <v>-0.113</v>
+        <v>-0.228</v>
       </c>
       <c r="AA359" s="10" t="inlineStr">
         <is>
@@ -28637,16 +28633,16 @@
         </is>
       </c>
       <c r="U383" s="11" t="n">
-        <v>3.56</v>
+        <v>3.79</v>
       </c>
       <c r="V383" s="12" t="n">
-        <v>337</v>
+        <v>359</v>
       </c>
       <c r="W383" s="6" t="n">
-        <v>93557</v>
+        <v>99601</v>
       </c>
       <c r="X383" s="12" t="n">
-        <v>8851409</v>
+        <v>9423270</v>
       </c>
       <c r="Y383" s="3" t="inlineStr">
         <is>
@@ -28654,7 +28650,7 @@
         </is>
       </c>
       <c r="Z383" s="13" t="n">
-        <v>-0.317</v>
+        <v>-0.359</v>
       </c>
       <c r="AA383" s="10" t="inlineStr">
         <is>
@@ -30385,16 +30381,16 @@
         </is>
       </c>
       <c r="U407" s="11" t="n">
-        <v>0.33</v>
+        <v>0.39</v>
       </c>
       <c r="V407" s="12" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="W407" s="6" t="n">
-        <v>1445</v>
+        <v>1708</v>
       </c>
       <c r="X407" s="12" t="n">
-        <v>136749</v>
+        <v>161613</v>
       </c>
       <c r="Y407" s="3" t="inlineStr">
         <is>
@@ -30402,7 +30398,7 @@
         </is>
       </c>
       <c r="Z407" s="14" t="n">
-        <v>1.068</v>
+        <v>0.75</v>
       </c>
       <c r="AA407" s="10" t="inlineStr">
         <is>
@@ -32181,16 +32177,16 @@
         </is>
       </c>
       <c r="U431" s="11" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="V431" s="12" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="W431" s="6" t="n">
-        <v>8935</v>
+        <v>10249</v>
       </c>
       <c r="X431" s="12" t="n">
-        <v>845359</v>
+        <v>969677</v>
       </c>
       <c r="Y431" s="3" t="inlineStr">
         <is>
@@ -32198,7 +32194,7 @@
         </is>
       </c>
       <c r="Z431" s="14" t="n">
-        <v>0.64</v>
+        <v>0.43</v>
       </c>
       <c r="AA431" s="10" t="inlineStr">
         <is>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -33961,16 +33953,16 @@
         </is>
       </c>
       <c r="U455" s="11" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="V455" s="12" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="W455" s="6" t="n">
-        <v>3679</v>
+        <v>4336</v>
       </c>
       <c r="X455" s="12" t="n">
-        <v>348089</v>
+        <v>410248</v>
       </c>
       <c r="Y455" s="3" t="inlineStr">
         <is>
@@ -33978,7 +33970,7 @@
         </is>
       </c>
       <c r="Z455" s="14" t="n">
-        <v>0.354</v>
+        <v>0.149</v>
       </c>
       <c r="AA455" s="10" t="inlineStr">
         <is>
@@ -35713,24 +35705,24 @@
         </is>
       </c>
       <c r="U479" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V479" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W479" s="6" t="n">
-        <v>22601</v>
+        <v>26017</v>
       </c>
       <c r="X479" s="12" t="n">
-        <v>2138262</v>
+        <v>2461487</v>
       </c>
       <c r="Y479" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z479" s="14" t="n">
-        <v>0.081</v>
+      <c r="Z479" s="13" t="n">
+        <v>-0.061</v>
       </c>
       <c r="AA479" s="10" t="inlineStr">
         <is>
@@ -35935,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39423,7 +39415,7 @@
       </c>
       <c r="S532" s="3" t="inlineStr">
         <is>
-          <t>eastus</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T532" s="3" t="inlineStr">
@@ -39449,7 +39441,7 @@
       </c>
       <c r="AA532" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -40841,24 +40833,24 @@
         </is>
       </c>
       <c r="U551" s="11" t="n">
-        <v>2.51</v>
+        <v>2.89</v>
       </c>
       <c r="V551" s="12" t="n">
-        <v>237</v>
+        <v>273</v>
       </c>
       <c r="W551" s="6" t="n">
-        <v>10994</v>
+        <v>12658</v>
       </c>
       <c r="X551" s="12" t="n">
-        <v>1040123</v>
+        <v>1197592</v>
       </c>
       <c r="Y551" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z551" s="14" t="n">
-        <v>0.112</v>
+      <c r="Z551" s="13" t="n">
+        <v>-0.035</v>
       </c>
       <c r="AA551" s="10" t="inlineStr">
         <is>
@@ -42633,16 +42625,16 @@
         </is>
       </c>
       <c r="U575" s="11" t="n">
-        <v>2.72</v>
+        <v>2.89</v>
       </c>
       <c r="V575" s="12" t="n">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="W575" s="6" t="n">
-        <v>71482</v>
+        <v>75949</v>
       </c>
       <c r="X575" s="12" t="n">
-        <v>6762874</v>
+        <v>7185554</v>
       </c>
       <c r="Y575" s="3" t="inlineStr">
         <is>
@@ -42650,7 +42642,7 @@
         </is>
       </c>
       <c r="Z575" s="13" t="n">
-        <v>-0.148</v>
+        <v>-0.198</v>
       </c>
       <c r="AA575" s="10" t="inlineStr">
         <is>
@@ -43039,7 +43031,7 @@
       </c>
       <c r="S580" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>westus2</t>
         </is>
       </c>
       <c r="T580" s="3" t="inlineStr">
@@ -43065,7 +43057,7 @@
       </c>
       <c r="AA580" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (westus2).</t>
         </is>
       </c>
     </row>
@@ -44457,16 +44449,16 @@
         </is>
       </c>
       <c r="U599" s="11" t="n">
-        <v>3.3</v>
+        <v>3.79</v>
       </c>
       <c r="V599" s="12" t="n">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="W599" s="6" t="n">
-        <v>14454</v>
+        <v>16600</v>
       </c>
       <c r="X599" s="12" t="n">
-        <v>1367493</v>
+        <v>1570545</v>
       </c>
       <c r="Y599" s="3" t="inlineStr">
         <is>
@@ -44474,7 +44466,7 @@
         </is>
       </c>
       <c r="Z599" s="13" t="n">
-        <v>-0.113</v>
+        <v>-0.228</v>
       </c>
       <c r="AA599" s="10" t="inlineStr">
         <is>
@@ -46221,16 +46213,16 @@
         </is>
       </c>
       <c r="U623" s="11" t="n">
-        <v>3.56</v>
+        <v>3.79</v>
       </c>
       <c r="V623" s="12" t="n">
-        <v>337</v>
+        <v>359</v>
       </c>
       <c r="W623" s="6" t="n">
-        <v>93557</v>
+        <v>99601</v>
       </c>
       <c r="X623" s="12" t="n">
-        <v>8851409</v>
+        <v>9423270</v>
       </c>
       <c r="Y623" s="3" t="inlineStr">
         <is>
@@ -46238,7 +46230,7 @@
         </is>
       </c>
       <c r="Z623" s="13" t="n">
-        <v>-0.317</v>
+        <v>-0.359</v>
       </c>
       <c r="AA623" s="10" t="inlineStr">
         <is>
@@ -47969,16 +47961,16 @@
         </is>
       </c>
       <c r="U647" s="11" t="n">
-        <v>0.33</v>
+        <v>0.39</v>
       </c>
       <c r="V647" s="12" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="W647" s="6" t="n">
-        <v>1445</v>
+        <v>1708</v>
       </c>
       <c r="X647" s="12" t="n">
-        <v>136749</v>
+        <v>161613</v>
       </c>
       <c r="Y647" s="3" t="inlineStr">
         <is>
@@ -47986,7 +47978,7 @@
         </is>
       </c>
       <c r="Z647" s="14" t="n">
-        <v>1.068</v>
+        <v>0.75</v>
       </c>
       <c r="AA647" s="10" t="inlineStr">
         <is>
@@ -49765,16 +49757,16 @@
         </is>
       </c>
       <c r="U671" s="11" t="n">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="V671" s="12" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="W671" s="6" t="n">
-        <v>8935</v>
+        <v>10249</v>
       </c>
       <c r="X671" s="12" t="n">
-        <v>845359</v>
+        <v>969677</v>
       </c>
       <c r="Y671" s="3" t="inlineStr">
         <is>
@@ -49782,7 +49774,7 @@
         </is>
       </c>
       <c r="Z671" s="14" t="n">
-        <v>0.64</v>
+        <v>0.43</v>
       </c>
       <c r="AA671" s="10" t="inlineStr">
         <is>
@@ -51541,16 +51533,16 @@
         </is>
       </c>
       <c r="U695" s="11" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="V695" s="12" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="W695" s="6" t="n">
-        <v>3679</v>
+        <v>4336</v>
       </c>
       <c r="X695" s="12" t="n">
-        <v>348089</v>
+        <v>410248</v>
       </c>
       <c r="Y695" s="3" t="inlineStr">
         <is>
@@ -51558,7 +51550,7 @@
         </is>
       </c>
       <c r="Z695" s="14" t="n">
-        <v>0.354</v>
+        <v>0.149</v>
       </c>
       <c r="AA695" s="10" t="inlineStr">
         <is>
@@ -53293,24 +53285,24 @@
         </is>
       </c>
       <c r="U719" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V719" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W719" s="6" t="n">
-        <v>22601</v>
+        <v>26017</v>
       </c>
       <c r="X719" s="12" t="n">
-        <v>2138262</v>
+        <v>2461487</v>
       </c>
       <c r="Y719" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z719" s="14" t="n">
-        <v>0.081</v>
+      <c r="Z719" s="13" t="n">
+        <v>-0.061</v>
       </c>
       <c r="AA719" s="10" t="inlineStr">
         <is>
@@ -53687,7 +53679,7 @@
       </c>
       <c r="S724" s="3" t="inlineStr">
         <is>
-          <t>eastus</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T724" s="3" t="inlineStr">
@@ -53711,7 +53703,7 @@
       <c r="Z724" s="3" t="n"/>
       <c r="AA724" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -55077,16 +55069,16 @@
         </is>
       </c>
       <c r="U743" s="11" t="n">
-        <v>2.51</v>
+        <v>2.89</v>
       </c>
       <c r="V743" s="12" t="n">
-        <v>237</v>
+        <v>273</v>
       </c>
       <c r="W743" s="6" t="n">
-        <v>10994</v>
+        <v>12658</v>
       </c>
       <c r="X743" s="12" t="n">
-        <v>1040123</v>
+        <v>1197592</v>
       </c>
       <c r="Y743" s="3" t="inlineStr">
         <is>
@@ -55094,7 +55086,7 @@
         </is>
       </c>
       <c r="Z743" s="13" t="n">
-        <v>-0.029</v>
+        <v>-0.157</v>
       </c>
       <c r="AA743" s="10" t="inlineStr">
         <is>
@@ -56869,16 +56861,16 @@
         </is>
       </c>
       <c r="U767" s="11" t="n">
-        <v>2.72</v>
+        <v>2.89</v>
       </c>
       <c r="V767" s="12" t="n">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="W767" s="6" t="n">
-        <v>71482</v>
+        <v>75949</v>
       </c>
       <c r="X767" s="12" t="n">
-        <v>6762874</v>
+        <v>7185554</v>
       </c>
       <c r="Y767" s="3" t="inlineStr">
         <is>
@@ -56886,7 +56878,7 @@
         </is>
       </c>
       <c r="Z767" s="13" t="n">
-        <v>-0.256</v>
+        <v>-0.3</v>
       </c>
       <c r="AA767" s="10" t="inlineStr">
         <is>
@@ -57259,7 +57251,7 @@
       </c>
       <c r="S772" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>westus2</t>
         </is>
       </c>
       <c r="T772" s="3" t="inlineStr">
@@ -57283,7 +57275,7 @@
       <c r="Z772" s="3" t="n"/>
       <c r="AA772" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (westus2).</t>
         </is>
       </c>
     </row>
@@ -58649,16 +58641,16 @@
         </is>
       </c>
       <c r="U791" s="11" t="n">
-        <v>3.3</v>
+        <v>3.79</v>
       </c>
       <c r="V791" s="12" t="n">
-        <v>312</v>
+        <v>359</v>
       </c>
       <c r="W791" s="6" t="n">
-        <v>14454</v>
+        <v>16600</v>
       </c>
       <c r="X791" s="12" t="n">
-        <v>1367493</v>
+        <v>1570545</v>
       </c>
       <c r="Y791" s="3" t="inlineStr">
         <is>
@@ -58666,7 +58658,7 @@
         </is>
       </c>
       <c r="Z791" s="13" t="n">
-        <v>-0.179</v>
+        <v>-0.285</v>
       </c>
       <c r="AA791" s="10" t="inlineStr">
         <is>
@@ -60413,16 +60405,16 @@
         </is>
       </c>
       <c r="U815" s="11" t="n">
-        <v>3.56</v>
+        <v>3.79</v>
       </c>
       <c r="V815" s="12" t="n">
-        <v>337</v>
+        <v>359</v>
       </c>
       <c r="W815" s="6" t="n">
-        <v>93557</v>
+        <v>99601</v>
       </c>
       <c r="X815" s="12" t="n">
-        <v>8851409</v>
+        <v>9423270</v>
       </c>
       <c r="Y815" s="3" t="inlineStr">
         <is>
@@ -60430,7 +60422,7 @@
         </is>
       </c>
       <c r="Z815" s="13" t="n">
-        <v>-0.368</v>
+        <v>-0.406</v>
       </c>
       <c r="AA815" s="10" t="inlineStr">
         <is>
@@ -62147,24 +62139,24 @@
         </is>
       </c>
       <c r="U839" s="11" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="V839" s="12" t="n">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="W839" s="6" t="n">
-        <v>3679</v>
+        <v>4336</v>
       </c>
       <c r="X839" s="12" t="n">
-        <v>348089</v>
+        <v>410248</v>
       </c>
       <c r="Y839" s="3" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z839" s="14" t="n">
-        <v>0.005</v>
+      <c r="Z839" s="13" t="n">
+        <v>-0.148</v>
       </c>
       <c r="AA839" s="10" t="inlineStr">
         <is>
@@ -63899,16 +63891,16 @@
         </is>
       </c>
       <c r="U863" s="11" t="n">
-        <v>0.86</v>
+        <v>0.99</v>
       </c>
       <c r="V863" s="12" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="W863" s="6" t="n">
-        <v>22601</v>
+        <v>26017</v>
       </c>
       <c r="X863" s="12" t="n">
-        <v>2138262</v>
+        <v>2461487</v>
       </c>
       <c r="Y863" s="3" t="inlineStr">
         <is>
@@ -63916,7 +63908,7 @@
         </is>
       </c>
       <c r="Z863" s="13" t="n">
-        <v>-0.185</v>
+        <v>-0.292</v>
       </c>
       <c r="AA863" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-17
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -4255,7 +4255,7 @@
       </c>
       <c r="S52" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>eastus</t>
         </is>
       </c>
       <c r="T52" s="3" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="AA52" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (eastus).</t>
         </is>
       </c>
     </row>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="S100" s="3" t="inlineStr">
         <is>
-          <t>westus2</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T100" s="3" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="AA100" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (westus2).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -21835,7 +21835,7 @@
       </c>
       <c r="S292" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>eastus</t>
         </is>
       </c>
       <c r="T292" s="3" t="inlineStr">
@@ -21861,7 +21861,7 @@
       </c>
       <c r="AA292" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (eastus).</t>
         </is>
       </c>
     </row>
@@ -25451,7 +25451,7 @@
       </c>
       <c r="S340" s="3" t="inlineStr">
         <is>
-          <t>westus2</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T340" s="3" t="inlineStr">
@@ -25477,7 +25477,7 @@
       </c>
       <c r="AA340" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (westus2).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -39415,7 +39415,7 @@
       </c>
       <c r="S532" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>eastus</t>
         </is>
       </c>
       <c r="T532" s="3" t="inlineStr">
@@ -39441,7 +39441,7 @@
       </c>
       <c r="AA532" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (eastus).</t>
         </is>
       </c>
     </row>
@@ -43031,7 +43031,7 @@
       </c>
       <c r="S580" s="3" t="inlineStr">
         <is>
-          <t>westus2</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T580" s="3" t="inlineStr">
@@ -43057,7 +43057,7 @@
       </c>
       <c r="AA580" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (westus2).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>
@@ -53679,7 +53679,7 @@
       </c>
       <c r="S724" s="3" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>eastus</t>
         </is>
       </c>
       <c r="T724" s="3" t="inlineStr">
@@ -53703,7 +53703,7 @@
       <c r="Z724" s="3" t="n"/>
       <c r="AA724" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (eastus2).</t>
+          <t>No India SKU; used US region (eastus).</t>
         </is>
       </c>
     </row>
@@ -57251,7 +57251,7 @@
       </c>
       <c r="S772" s="3" t="inlineStr">
         <is>
-          <t>westus2</t>
+          <t>eastus2</t>
         </is>
       </c>
       <c r="T772" s="3" t="inlineStr">
@@ -57275,7 +57275,7 @@
       <c r="Z772" s="3" t="n"/>
       <c r="AA772" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used US region (westus2).</t>
+          <t>No India SKU; used US region (eastus2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-18
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-19
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-20
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-23
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-25
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-26
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-27
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-07-28
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-02
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-03
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-04
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-05
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -11681,10 +11681,10 @@
         </is>
       </c>
       <c r="U151" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V151" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W151" s="9" t="n"/>
       <c r="X151" s="8" t="n"/>
@@ -11694,7 +11694,7 @@
         </is>
       </c>
       <c r="Z151" s="14" t="n">
-        <v>1.846</v>
+        <v>1.265</v>
       </c>
       <c r="AA151" s="10" t="inlineStr">
         <is>
@@ -12801,16 +12801,16 @@
         </is>
       </c>
       <c r="U167" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V167" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W167" s="6" t="n">
-        <v>1708</v>
+        <v>2146</v>
       </c>
       <c r="X167" s="12" t="n">
-        <v>161613</v>
+        <v>203052</v>
       </c>
       <c r="Y167" s="3" t="inlineStr">
         <is>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="Z167" s="14" t="n">
-        <v>0.75</v>
+        <v>0.392</v>
       </c>
       <c r="AA167" s="10" t="inlineStr">
         <is>
@@ -14597,16 +14597,16 @@
         </is>
       </c>
       <c r="U191" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V191" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W191" s="6" t="n">
-        <v>10249</v>
+        <v>12877</v>
       </c>
       <c r="X191" s="12" t="n">
-        <v>969677</v>
+        <v>1218312</v>
       </c>
       <c r="Y191" s="3" t="inlineStr">
         <is>
@@ -14614,7 +14614,7 @@
         </is>
       </c>
       <c r="Z191" s="14" t="n">
-        <v>0.43</v>
+        <v>0.138</v>
       </c>
       <c r="AA191" s="10" t="inlineStr">
         <is>
@@ -18698,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -29265,10 +29265,10 @@
         </is>
       </c>
       <c r="U391" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V391" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W391" s="9" t="n"/>
       <c r="X391" s="8" t="n"/>
@@ -29278,7 +29278,7 @@
         </is>
       </c>
       <c r="Z391" s="14" t="n">
-        <v>1.846</v>
+        <v>1.265</v>
       </c>
       <c r="AA391" s="10" t="inlineStr">
         <is>
@@ -30385,16 +30385,16 @@
         </is>
       </c>
       <c r="U407" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V407" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W407" s="6" t="n">
-        <v>1708</v>
+        <v>2146</v>
       </c>
       <c r="X407" s="12" t="n">
-        <v>161613</v>
+        <v>203052</v>
       </c>
       <c r="Y407" s="3" t="inlineStr">
         <is>
@@ -30402,7 +30402,7 @@
         </is>
       </c>
       <c r="Z407" s="14" t="n">
-        <v>0.75</v>
+        <v>0.392</v>
       </c>
       <c r="AA407" s="10" t="inlineStr">
         <is>
@@ -32181,16 +32181,16 @@
         </is>
       </c>
       <c r="U431" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V431" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W431" s="6" t="n">
-        <v>10249</v>
+        <v>12877</v>
       </c>
       <c r="X431" s="12" t="n">
-        <v>969677</v>
+        <v>1218312</v>
       </c>
       <c r="Y431" s="3" t="inlineStr">
         <is>
@@ -32198,7 +32198,7 @@
         </is>
       </c>
       <c r="Z431" s="14" t="n">
-        <v>0.43</v>
+        <v>0.138</v>
       </c>
       <c r="AA431" s="10" t="inlineStr">
         <is>
@@ -36282,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -46849,10 +46849,10 @@
         </is>
       </c>
       <c r="U631" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V631" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W631" s="9" t="n"/>
       <c r="X631" s="8" t="n"/>
@@ -46862,7 +46862,7 @@
         </is>
       </c>
       <c r="Z631" s="14" t="n">
-        <v>1.846</v>
+        <v>1.265</v>
       </c>
       <c r="AA631" s="10" t="inlineStr">
         <is>
@@ -47969,16 +47969,16 @@
         </is>
       </c>
       <c r="U647" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V647" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W647" s="6" t="n">
-        <v>1708</v>
+        <v>2146</v>
       </c>
       <c r="X647" s="12" t="n">
-        <v>161613</v>
+        <v>203052</v>
       </c>
       <c r="Y647" s="3" t="inlineStr">
         <is>
@@ -47986,7 +47986,7 @@
         </is>
       </c>
       <c r="Z647" s="14" t="n">
-        <v>0.75</v>
+        <v>0.392</v>
       </c>
       <c r="AA647" s="10" t="inlineStr">
         <is>
@@ -49765,16 +49765,16 @@
         </is>
       </c>
       <c r="U671" s="11" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="V671" s="12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="W671" s="6" t="n">
-        <v>10249</v>
+        <v>12877</v>
       </c>
       <c r="X671" s="12" t="n">
-        <v>969677</v>
+        <v>1218312</v>
       </c>
       <c r="Y671" s="3" t="inlineStr">
         <is>
@@ -49782,7 +49782,7 @@
         </is>
       </c>
       <c r="Z671" s="14" t="n">
-        <v>0.43</v>
+        <v>0.138</v>
       </c>
       <c r="AA671" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-06
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19230,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19703,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19770,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20275,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20342,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20815,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36219,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36814,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37287,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37354,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37859,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37926,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38399,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38466,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38971,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39038,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-07
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-09
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-10
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-12
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-13
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -18351,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18891,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18958,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19431,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19971,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20038,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20543,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20610,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21083,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21150,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -35935,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36475,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36542,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37015,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37082,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37555,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37622,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38194,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38667,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38734,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-14
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-15
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-16
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15368,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr"/>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15392,7 +15396,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18351,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18414,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18635,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18698,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18891,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18958,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19163,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19230,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19431,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19498,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19703,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19770,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19971,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20038,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20275,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20342,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20543,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20610,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20815,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20882,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21083,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21150,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21387,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21454,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32948,7 +32952,11 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr"/>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>atl</t>
+        </is>
+      </c>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32972,7 +32980,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region ().</t>
+          <t>No India SKU; used global/other region (atl).</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35935,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35998,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36219,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36282,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36475,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36542,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36814,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37015,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37082,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37287,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37354,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37555,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37622,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37859,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37926,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38127,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38194,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38399,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38466,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38667,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38734,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38971,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39038,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-17
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -15368,11 +15368,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S201" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S201" s="3" t="inlineStr"/>
       <c r="T201" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -15396,7 +15392,7 @@
       </c>
       <c r="AA201" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>
@@ -32952,11 +32948,7 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S441" s="3" t="inlineStr">
-        <is>
-          <t>atl</t>
-        </is>
-      </c>
+      <c r="S441" s="3" t="inlineStr"/>
       <c r="T441" s="3" t="inlineStr">
         <is>
           <t>global/other</t>
@@ -32980,7 +32972,7 @@
       </c>
       <c r="AA441" s="10" t="inlineStr">
         <is>
-          <t>No India SKU; used global/other region (atl).</t>
+          <t>No India SKU; used global/other region ().</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-18
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-22
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-23
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-24
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-25
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-27
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-28
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-29
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-30
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-08-31
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-02
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-03
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-04
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -15225,10 +15225,10 @@
         </is>
       </c>
       <c r="U199" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V199" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W199" s="9" t="n"/>
       <c r="X199" s="8" t="n"/>
@@ -15238,7 +15238,7 @@
         </is>
       </c>
       <c r="Z199" s="14" t="n">
-        <v>0.868</v>
+        <v>0.6970000000000001</v>
       </c>
       <c r="AA199" s="10" t="inlineStr">
         <is>
@@ -16373,16 +16373,16 @@
         </is>
       </c>
       <c r="U215" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V215" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W215" s="6" t="n">
-        <v>4336</v>
+        <v>4774</v>
       </c>
       <c r="X215" s="12" t="n">
-        <v>410248</v>
+        <v>451687</v>
       </c>
       <c r="Y215" s="3" t="inlineStr">
         <is>
@@ -16390,7 +16390,7 @@
         </is>
       </c>
       <c r="Z215" s="14" t="n">
-        <v>0.149</v>
+        <v>0.043</v>
       </c>
       <c r="AA215" s="10" t="inlineStr">
         <is>
@@ -18125,16 +18125,16 @@
         </is>
       </c>
       <c r="U239" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V239" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W239" s="6" t="n">
-        <v>26017</v>
+        <v>28645</v>
       </c>
       <c r="X239" s="12" t="n">
-        <v>2461487</v>
+        <v>2710122</v>
       </c>
       <c r="Y239" s="3" t="inlineStr">
         <is>
@@ -18142,7 +18142,7 @@
         </is>
       </c>
       <c r="Z239" s="13" t="n">
-        <v>-0.061</v>
+        <v>-0.147</v>
       </c>
       <c r="AA239" s="10" t="inlineStr">
         <is>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -32805,10 +32805,10 @@
         </is>
       </c>
       <c r="U439" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V439" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W439" s="9" t="n"/>
       <c r="X439" s="8" t="n"/>
@@ -32818,7 +32818,7 @@
         </is>
       </c>
       <c r="Z439" s="14" t="n">
-        <v>0.868</v>
+        <v>0.6970000000000001</v>
       </c>
       <c r="AA439" s="10" t="inlineStr">
         <is>
@@ -33953,16 +33953,16 @@
         </is>
       </c>
       <c r="U455" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V455" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W455" s="6" t="n">
-        <v>4336</v>
+        <v>4774</v>
       </c>
       <c r="X455" s="12" t="n">
-        <v>410248</v>
+        <v>451687</v>
       </c>
       <c r="Y455" s="3" t="inlineStr">
         <is>
@@ -33970,7 +33970,7 @@
         </is>
       </c>
       <c r="Z455" s="14" t="n">
-        <v>0.149</v>
+        <v>0.043</v>
       </c>
       <c r="AA455" s="10" t="inlineStr">
         <is>
@@ -35705,16 +35705,16 @@
         </is>
       </c>
       <c r="U479" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V479" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W479" s="6" t="n">
-        <v>26017</v>
+        <v>28645</v>
       </c>
       <c r="X479" s="12" t="n">
-        <v>2461487</v>
+        <v>2710122</v>
       </c>
       <c r="Y479" s="3" t="inlineStr">
         <is>
@@ -35722,7 +35722,7 @@
         </is>
       </c>
       <c r="Z479" s="13" t="n">
-        <v>-0.061</v>
+        <v>-0.147</v>
       </c>
       <c r="AA479" s="10" t="inlineStr">
         <is>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $0.99/GPU/hr (₹94) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -50385,10 +50385,10 @@
         </is>
       </c>
       <c r="U679" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V679" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W679" s="9" t="n"/>
       <c r="X679" s="8" t="n"/>
@@ -50398,7 +50398,7 @@
         </is>
       </c>
       <c r="Z679" s="14" t="n">
-        <v>0.868</v>
+        <v>0.6970000000000001</v>
       </c>
       <c r="AA679" s="10" t="inlineStr">
         <is>
@@ -51533,16 +51533,16 @@
         </is>
       </c>
       <c r="U695" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V695" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W695" s="6" t="n">
-        <v>4336</v>
+        <v>4774</v>
       </c>
       <c r="X695" s="12" t="n">
-        <v>410248</v>
+        <v>451687</v>
       </c>
       <c r="Y695" s="3" t="inlineStr">
         <is>
@@ -51550,7 +51550,7 @@
         </is>
       </c>
       <c r="Z695" s="14" t="n">
-        <v>0.149</v>
+        <v>0.043</v>
       </c>
       <c r="AA695" s="10" t="inlineStr">
         <is>
@@ -53285,16 +53285,16 @@
         </is>
       </c>
       <c r="U719" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V719" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W719" s="6" t="n">
-        <v>26017</v>
+        <v>28645</v>
       </c>
       <c r="X719" s="12" t="n">
-        <v>2461487</v>
+        <v>2710122</v>
       </c>
       <c r="Y719" s="3" t="inlineStr">
         <is>
@@ -53302,7 +53302,7 @@
         </is>
       </c>
       <c r="Z719" s="13" t="n">
-        <v>-0.061</v>
+        <v>-0.147</v>
       </c>
       <c r="AA719" s="10" t="inlineStr">
         <is>
@@ -61003,10 +61003,10 @@
         </is>
       </c>
       <c r="U823" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V823" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W823" s="9" t="n"/>
       <c r="X823" s="8" t="n"/>
@@ -62139,16 +62139,16 @@
         </is>
       </c>
       <c r="U839" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V839" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W839" s="6" t="n">
-        <v>4336</v>
+        <v>4774</v>
       </c>
       <c r="X839" s="12" t="n">
-        <v>410248</v>
+        <v>451687</v>
       </c>
       <c r="Y839" s="3" t="inlineStr">
         <is>
@@ -62156,7 +62156,7 @@
         </is>
       </c>
       <c r="Z839" s="13" t="n">
-        <v>-0.148</v>
+        <v>-0.226</v>
       </c>
       <c r="AA839" s="10" t="inlineStr">
         <is>
@@ -63891,16 +63891,16 @@
         </is>
       </c>
       <c r="U863" s="11" t="n">
-        <v>0.99</v>
+        <v>1.09</v>
       </c>
       <c r="V863" s="12" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="W863" s="6" t="n">
-        <v>26017</v>
+        <v>28645</v>
       </c>
       <c r="X863" s="12" t="n">
-        <v>2461487</v>
+        <v>2710122</v>
       </c>
       <c r="Y863" s="3" t="inlineStr">
         <is>
@@ -63908,7 +63908,7 @@
         </is>
       </c>
       <c r="Z863" s="13" t="n">
-        <v>-0.292</v>
+        <v>-0.357</v>
       </c>
       <c r="AA863" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-06
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-07
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-08
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-09
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-11
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-14
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-15
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-17
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-18
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-19
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-20
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-22
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-24
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="Z35" s="3" t="n"/>
       <c r="AA35" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       <c r="Z38" s="3" t="n"/>
       <c r="AA38" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       <c r="Z39" s="3" t="n"/>
       <c r="AA39" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="Z42" s="3" t="n"/>
       <c r="AA42" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="Z43" s="3" t="n"/>
       <c r="AA43" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
       <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       <c r="Z47" s="3" t="n"/>
       <c r="AA47" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       <c r="Z242" s="3" t="n"/>
       <c r="AA242" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18410,7 +18410,7 @@
       <c r="Z243" s="3" t="n"/>
       <c r="AA243" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -18631,7 +18631,7 @@
       <c r="Z246" s="3" t="n"/>
       <c r="AA246" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18694,7 +18694,7 @@
       <c r="Z247" s="3" t="n"/>
       <c r="AA247" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       <c r="Z250" s="3" t="n"/>
       <c r="AA250" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -18954,7 +18954,7 @@
       <c r="Z251" s="3" t="n"/>
       <c r="AA251" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19159,7 +19159,7 @@
       <c r="Z254" s="3" t="n"/>
       <c r="AA254" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19226,7 +19226,7 @@
       <c r="Z255" s="3" t="n"/>
       <c r="AA255" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19427,7 +19427,7 @@
       <c r="Z258" s="3" t="n"/>
       <c r="AA258" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       <c r="Z259" s="3" t="n"/>
       <c r="AA259" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19699,7 @@
       <c r="Z262" s="3" t="n"/>
       <c r="AA262" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       <c r="Z263" s="3" t="n"/>
       <c r="AA263" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       <c r="Z266" s="3" t="n"/>
       <c r="AA266" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20034,7 +20034,7 @@
       <c r="Z267" s="3" t="n"/>
       <c r="AA267" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20271,7 +20271,7 @@
       <c r="Z270" s="3" t="n"/>
       <c r="AA270" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="Z271" s="3" t="n"/>
       <c r="AA271" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20539,7 +20539,7 @@
       <c r="Z274" s="3" t="n"/>
       <c r="AA274" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -20606,7 +20606,7 @@
       <c r="Z275" s="3" t="n"/>
       <c r="AA275" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -20811,7 +20811,7 @@
       <c r="Z278" s="3" t="n"/>
       <c r="AA278" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -20878,7 +20878,7 @@
       <c r="Z279" s="3" t="n"/>
       <c r="AA279" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       <c r="Z282" s="3" t="n"/>
       <c r="AA282" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
         </is>
       </c>
     </row>
@@ -21146,7 +21146,7 @@
       <c r="Z283" s="3" t="n"/>
       <c r="AA283" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
         </is>
       </c>
     </row>
@@ -21383,7 +21383,7 @@
       <c r="Z286" s="3" t="n"/>
       <c r="AA286" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -21450,7 +21450,7 @@
       <c r="Z287" s="3" t="n"/>
       <c r="AA287" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -35927,7 +35927,7 @@
       <c r="Z482" s="3" t="n"/>
       <c r="AA482" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -35990,7 +35990,7 @@
       <c r="Z483" s="3" t="n"/>
       <c r="AA483" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36211,7 +36211,7 @@
       <c r="Z486" s="3" t="n"/>
       <c r="AA486" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36274,7 +36274,7 @@
       <c r="Z487" s="3" t="n"/>
       <c r="AA487" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
       <c r="Z490" s="3" t="n"/>
       <c r="AA490" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -36534,7 +36534,7 @@
       <c r="Z491" s="3" t="n"/>
       <c r="AA491" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       <c r="Z494" s="3" t="n"/>
       <c r="AA494" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       <c r="Z495" s="3" t="n"/>
       <c r="AA495" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37007,7 +37007,7 @@
       <c r="Z498" s="3" t="n"/>
       <c r="AA498" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37074,7 +37074,7 @@
       <c r="Z499" s="3" t="n"/>
       <c r="AA499" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37279,7 +37279,7 @@
       <c r="Z502" s="3" t="n"/>
       <c r="AA502" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       <c r="Z503" s="3" t="n"/>
       <c r="AA503" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37547,7 +37547,7 @@
       <c r="Z506" s="3" t="n"/>
       <c r="AA506" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -37614,7 +37614,7 @@
       <c r="Z507" s="3" t="n"/>
       <c r="AA507" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -37851,7 +37851,7 @@
       <c r="Z510" s="3" t="n"/>
       <c r="AA510" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -37918,7 +37918,7 @@
       <c r="Z511" s="3" t="n"/>
       <c r="AA511" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38119,7 +38119,7 @@
       <c r="Z514" s="3" t="n"/>
       <c r="AA514" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38186,7 +38186,7 @@
       <c r="Z515" s="3" t="n"/>
       <c r="AA515" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38391,7 +38391,7 @@
       <c r="Z518" s="3" t="n"/>
       <c r="AA518" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38458,7 +38458,7 @@
       <c r="Z519" s="3" t="n"/>
       <c r="AA519" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -38659,7 +38659,7 @@
       <c r="Z522" s="3" t="n"/>
       <c r="AA522" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.15/GPU/hr (₹298) [India region].</t>
         </is>
       </c>
     </row>
@@ -38726,7 +38726,7 @@
       <c r="Z523" s="3" t="n"/>
       <c r="AA523" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.12xlarge (L40S, 48 vCPU, 384GB RAM) at $3.94/GPU/hr (₹373) [India region].</t>
         </is>
       </c>
     </row>
@@ -38963,7 +38963,7 @@
       <c r="Z526" s="3" t="n"/>
       <c r="AA526" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -39030,7 +39030,7 @@
       <c r="Z527" s="3" t="n"/>
       <c r="AA527" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily pricing refresh 2026-09-26
</commit_message>
<xml_diff>
--- a/Neysa_Competitor_SKU_Match.xlsx
+++ b/Neysa_Competitor_SKU_Match.xlsx
@@ -767,7 +767,7 @@
       <c r="Z2" s="3" t="n"/>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       <c r="Z15" s="3" t="n"/>
       <c r="AA15" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       <c r="Z18" s="3" t="n"/>
       <c r="AA18" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       <c r="Z19" s="3" t="n"/>
       <c r="AA19" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       <c r="Z23" s="3" t="n"/>
       <c r="AA23" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $8.26/GPU/hr (₹781) [India region].</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="10" t="inlineStr">
         <is>
-          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $3.13/GPU/hr (₹296) [India region].</t>
+          <t>AWS SageMaker does not offer H100 NVL. Nearest: ml.p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) at $9.49/GPU/hr (₹898) [India region].</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       <c r="Z30" s="3" t="n"/>
       <c r="AA30" s="10" t="inlineStr">
         <is>
-          <t>OCI does not offer H100 NVL. Nearest: Oracle Compute Cloud@Customer - Compute - GPU.L40S - Resource Commit (L40S) at $0.60/GPU/hr (₹57) [global/other region].</t>
+          <t>OCI does not offer H100 NVL. Nearest: Oracle Cloud Infrastructure - Compute - GPU - H100 (H100 SXM) at $10.00/GPU/hr (₹946) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       <c r="Z31" s="3" t="n"/>
       <c r="AA31" s="10" t="inlineStr">
         <is>
-          <t>RunPod does not offer H100 NVL. Nearest: L40S (L40S) at $1.09/GPU/hr (₹103) [global/other region].</t>
+          <t>RunPod does not offer H100 NVL. Nearest: H100 PCIe (H100 SXM) at $2.89/GPU/hr (₹273) [global/other region].</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       <c r="Z34" s="3" t="n"/>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>AWS EC2 does not offer H100 NVL. Nearest: g6e.xlarge (L40S, 4 vCPU, 32GB RAM) at $2.23/GPU/hr (₹211) [India region].</t>
+          <t>AWS EC2 does not offer H100 NVL. Nearest: p5.48xlarge (H100 SXM, 192 vCPU, 2048GB RAM) 